<commit_message>
Fix product prices from site
</commit_message>
<xml_diff>
--- a/outputs/bushido_yandex_products.xlsx
+++ b/outputs/bushido_yandex_products.xlsx
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>50</v>
+        <v>160</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>50</v>
+        <v>160</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1546,7 +1546,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>50</v>
+        <v>1200</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1663,7 +1663,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>50</v>
+        <v>440</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>50</v>
+        <v>420</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>50</v>
+        <v>290</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>50</v>
+        <v>560</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>50</v>
+        <v>780</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>50</v>
+        <v>280</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>50</v>
+        <v>670</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>50</v>
+        <v>280</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>50</v>
+        <v>470</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>50</v>
+        <v>580</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>50</v>
+        <v>730</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>50</v>
+        <v>220</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>50</v>
+        <v>380</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>50</v>
+        <v>380</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2677,7 +2677,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>50</v>
+        <v>680</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -2716,7 +2716,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>50</v>
+        <v>620</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2755,7 +2755,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>50</v>
+        <v>620</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>50</v>
+        <v>800</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>50</v>
+        <v>800</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -2872,7 +2872,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>50</v>
+        <v>680</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2950,7 +2950,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>50</v>
+        <v>490</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>50</v>
+        <v>690</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>50</v>
+        <v>590</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3106,7 +3106,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3184,7 +3184,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>50</v>
+        <v>280</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>50</v>
+        <v>490</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -3301,7 +3301,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>50</v>
+        <v>370</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>50</v>
+        <v>420</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>50</v>
+        <v>310</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>50</v>
+        <v>290</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3496,7 +3496,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -3535,7 +3535,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -3574,7 +3574,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>50</v>
+        <v>600</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -3613,7 +3613,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>50</v>
+        <v>370</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>50</v>
+        <v>570</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -3691,7 +3691,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>50</v>
+        <v>220</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -3730,7 +3730,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>50</v>
+        <v>440</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>50</v>
+        <v>520</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>50</v>
+        <v>570</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -3886,7 +3886,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>50</v>
+        <v>440</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -3964,7 +3964,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -4003,7 +4003,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>50</v>
+        <v>270</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -4042,7 +4042,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -4081,7 +4081,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -4120,7 +4120,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>50</v>
+        <v>510</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -4159,7 +4159,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>50</v>
+        <v>440</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>50</v>
+        <v>600</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>50</v>
+        <v>460</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -4276,7 +4276,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -4315,7 +4315,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -4393,7 +4393,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -4432,7 +4432,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>50</v>
+        <v>490</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -4471,7 +4471,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>50</v>
+        <v>420</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -4510,7 +4510,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -4549,7 +4549,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>50</v>
+        <v>230</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -4627,7 +4627,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>50</v>
+        <v>470</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -4666,7 +4666,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>50</v>
+        <v>470</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -4744,7 +4744,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -4783,7 +4783,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>50</v>
+        <v>590</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -4822,7 +4822,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>50</v>
+        <v>440</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -4861,7 +4861,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>50</v>
+        <v>330</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -4900,7 +4900,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>50</v>
+        <v>580</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -4939,7 +4939,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -4978,7 +4978,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>50</v>
+        <v>280</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>50</v>
+        <v>2900</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -5095,7 +5095,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>50</v>
+        <v>3300</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -5134,7 +5134,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>50</v>
+        <v>420</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>50</v>
+        <v>2400</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -5251,7 +5251,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -5290,7 +5290,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>50</v>
+        <v>2650</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>50</v>
+        <v>2400</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -5368,7 +5368,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>50</v>
+        <v>3600</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>50</v>
+        <v>2700</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -5446,7 +5446,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>50</v>
+        <v>2000</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>50</v>
+        <v>2300</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -5524,7 +5524,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>50</v>
+        <v>1840</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -5563,7 +5563,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>50</v>
+        <v>1600</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -5602,7 +5602,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>50</v>
+        <v>2200</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -5641,7 +5641,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>50</v>
+        <v>1500</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -5680,7 +5680,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>50</v>
+        <v>2800</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -5719,7 +5719,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>50</v>
+        <v>1300</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -5758,7 +5758,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>50</v>
+        <v>2600</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -5797,7 +5797,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>50</v>
+        <v>4000</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>50</v>
+        <v>1550</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -5875,7 +5875,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>50</v>
+        <v>2500</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -5914,7 +5914,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>50</v>
+        <v>280</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -5953,7 +5953,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -5992,7 +5992,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>50</v>
+        <v>370</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -6031,7 +6031,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -6070,7 +6070,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -6109,7 +6109,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -6226,7 +6226,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>50</v>
+        <v>260</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -6265,7 +6265,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>50</v>
+        <v>260</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -6304,7 +6304,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>50</v>
+        <v>580</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -6343,7 +6343,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>50</v>
+        <v>520</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>50</v>
+        <v>450</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -6460,7 +6460,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>50</v>
+        <v>530</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -6499,7 +6499,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>50</v>
+        <v>370</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -6577,7 +6577,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>50</v>
+        <v>1480</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -6616,7 +6616,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>50</v>
+        <v>520</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>50</v>
+        <v>510</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -6694,7 +6694,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>50</v>
+        <v>980</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -6733,7 +6733,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>50</v>
+        <v>950</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -6772,7 +6772,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -6811,7 +6811,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>50</v>
+        <v>600</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -6850,7 +6850,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>50</v>
+        <v>850</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -6889,7 +6889,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>50</v>
+        <v>410</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -6928,7 +6928,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>50</v>
+        <v>950</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -6967,7 +6967,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>50</v>
+        <v>580</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -7006,7 +7006,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>50</v>
+        <v>630</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -7045,7 +7045,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>50</v>
+        <v>650</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -7084,7 +7084,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>50</v>
+        <v>570</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>50</v>
+        <v>340</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>50</v>
+        <v>170</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -7201,7 +7201,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -7240,7 +7240,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>50</v>
+        <v>290</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -7279,7 +7279,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -7318,7 +7318,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>50</v>
+        <v>450</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -7357,7 +7357,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>50</v>
+        <v>260</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -7396,7 +7396,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>50</v>
+        <v>270</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>50</v>
+        <v>950</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -7513,7 +7513,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>50</v>
+        <v>660</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -7552,7 +7552,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>50</v>
+        <v>370</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -7591,7 +7591,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -7630,7 +7630,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>50</v>
+        <v>540</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -7669,7 +7669,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>50</v>
+        <v>420</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>50</v>
+        <v>560</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -7747,7 +7747,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>50</v>
+        <v>540</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -7786,7 +7786,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>50</v>
+        <v>820</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -7825,7 +7825,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>50</v>
+        <v>800</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -7864,7 +7864,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -7903,7 +7903,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>50</v>
+        <v>650</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -7942,7 +7942,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>50</v>
+        <v>850</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -7981,7 +7981,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>50</v>
+        <v>280</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -8020,7 +8020,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>50</v>
+        <v>490</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -8059,7 +8059,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>50</v>
+        <v>270</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -8098,7 +8098,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -8137,7 +8137,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>50</v>
+        <v>830</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -8176,7 +8176,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -8215,7 +8215,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>50</v>
+        <v>890</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -8254,7 +8254,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -8293,7 +8293,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>50</v>
+        <v>840</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -8332,7 +8332,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>50</v>
+        <v>680</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -8371,7 +8371,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>50</v>
+        <v>1600</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -8410,7 +8410,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>50</v>
+        <v>1150</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -8449,7 +8449,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>50</v>
+        <v>950</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -8488,7 +8488,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>50</v>
+        <v>740</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -8527,7 +8527,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -8566,7 +8566,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>50</v>
+        <v>730</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -8605,7 +8605,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>50</v>
+        <v>310</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -8644,7 +8644,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>50</v>
+        <v>460</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -8683,7 +8683,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>50</v>
+        <v>420</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -8722,7 +8722,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>50</v>
+        <v>610</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -8761,7 +8761,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -8800,7 +8800,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -8839,7 +8839,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>50</v>
+        <v>720</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -8878,7 +8878,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>50</v>
+        <v>600</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -8917,7 +8917,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>50</v>
+        <v>620</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -8956,7 +8956,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>50</v>
+        <v>680</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -8995,7 +8995,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>50</v>
+        <v>1700</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -9034,7 +9034,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>50</v>
+        <v>1200</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>50</v>
+        <v>860</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -9112,7 +9112,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>50</v>
+        <v>1250</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -9151,7 +9151,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>50</v>
+        <v>790</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -9190,7 +9190,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>50</v>
+        <v>850</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -9229,7 +9229,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>50</v>
+        <v>1750</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -9268,7 +9268,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>50</v>
+        <v>1900</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -9307,7 +9307,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>50</v>
+        <v>420</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -9346,7 +9346,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -9385,7 +9385,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>50</v>
+        <v>270</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -9424,7 +9424,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>50</v>
+        <v>570</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -9463,7 +9463,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -9502,7 +9502,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>50</v>
+        <v>290</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -9541,7 +9541,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -9580,7 +9580,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>50</v>
+        <v>670</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -9619,7 +9619,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -9658,7 +9658,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -9697,7 +9697,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>50</v>
+        <v>170</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -9736,7 +9736,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -9775,7 +9775,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -9814,7 +9814,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>50</v>
+        <v>450</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -9853,7 +9853,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -9892,7 +9892,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -9931,7 +9931,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>50</v>
+        <v>600</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -9970,7 +9970,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -10360,7 +10360,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -10399,7 +10399,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>50</v>
+        <v>270</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -10477,7 +10477,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -10555,7 +10555,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>50</v>
+        <v>230</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -10594,7 +10594,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>50</v>
+        <v>230</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -10672,7 +10672,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -10711,7 +10711,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -10750,7 +10750,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>50</v>
+        <v>210</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -10789,7 +10789,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -10828,7 +10828,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -10867,7 +10867,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -10906,7 +10906,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -10945,7 +10945,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -10984,7 +10984,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -11023,7 +11023,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -11101,7 +11101,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -11179,7 +11179,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>50</v>
+        <v>105</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -11218,7 +11218,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -11257,7 +11257,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -11296,7 +11296,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -11335,7 +11335,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -11374,7 +11374,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -11413,7 +11413,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -11452,7 +11452,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -11491,7 +11491,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -11530,7 +11530,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>50</v>
+        <v>260</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>50</v>
+        <v>260</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>

</xml_diff>